<commit_message>
PARKEN.CO PP&E + Excel
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/PARKEN.CO.xlsx
+++ b/data/cox_xlsx/PARKEN.CO.xlsx
@@ -13816,15 +13816,39 @@
       <c r="N72" s="15">
         <v>2032.06</v>
       </c>
-      <c r="O72" s="16"/>
-      <c r="P72" s="16"/>
-      <c r="Q72" s="16"/>
-      <c r="R72" s="16"/>
-      <c r="S72" s="16"/>
-      <c r="T72" s="16"/>
-      <c r="U72" s="16"/>
+      <c r="O72" s="24">
+        <f t="shared" ref="O72:U72" si="1">O74+O75+O76+O77+O82+O84+O39</f>
+        <v>2010.11</v>
+      </c>
+      <c r="P72" s="24">
+        <f t="shared" si="1"/>
+        <v>2115.11</v>
+      </c>
+      <c r="Q72" s="24">
+        <f t="shared" si="1"/>
+        <v>2228.4</v>
+      </c>
+      <c r="R72" s="24">
+        <f t="shared" si="1"/>
+        <v>541.6</v>
+      </c>
+      <c r="S72" s="24">
+        <f t="shared" si="1"/>
+        <v>423.77</v>
+      </c>
+      <c r="T72" s="24">
+        <f t="shared" si="1"/>
+        <v>726.76</v>
+      </c>
+      <c r="U72" s="24">
+        <f t="shared" si="1"/>
+        <v>681.92</v>
+      </c>
       <c r="V72" s="16"/>
-      <c r="W72" s="16"/>
+      <c r="W72" s="16">
+        <f>SUM(W74:W79)</f>
+        <v>1.46</v>
+      </c>
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="14" t="s">
@@ -14027,7 +14051,10 @@
       <c r="O76" s="15">
         <v>923.37</v>
       </c>
-      <c r="P76" s="16"/>
+      <c r="P76" s="16">
+        <f>(O76+Q76)/2</f>
+        <v>939.17</v>
+      </c>
       <c r="Q76" s="15">
         <v>954.97</v>
       </c>

</xml_diff>